<commit_message>
graphes burndown burnup modifiés
</commit_message>
<xml_diff>
--- a/docs/pilotage/burndown-burnup.xlsx
+++ b/docs/pilotage/burndown-burnup.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/chaima/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{02450362-E4EF-5142-8919-2CD2785DA932}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{123845B6-2DBC-5742-B46E-1D39DE582447}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="140" yWindow="680" windowWidth="28480" windowHeight="16180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3480" yWindow="800" windowWidth="16360" windowHeight="16180" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Mode d'emploi" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="62">
   <si>
     <t>Modèle : Burndown de sprint &amp; Burnup de projet</t>
   </si>
@@ -142,9 +142,6 @@
     <t>S0</t>
   </si>
   <si>
-    <t>Départ</t>
-  </si>
-  <si>
     <t>S1</t>
   </si>
   <si>
@@ -187,32 +184,50 @@
     <t>Astuce : les indicateurs pointent sur la dernière ligne (S6). Si vous ajoutez des sprints, insérez les lignes AU-DESSUS de la dernière pour que les plages suivent.</t>
   </si>
   <si>
-    <t>Auth + inscription</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Upload PDF Terminé </t>
-  </si>
-  <si>
-    <t>Génération quiz terminée</t>
-  </si>
-  <si>
-    <t>Projet en cours</t>
-  </si>
-  <si>
-    <t>+20 : accessibilité RGAA + i18n exigées</t>
-  </si>
-  <si>
-    <t>+20: statisqtiques enseignant</t>
-  </si>
-  <si>
     <t>Réel (modifié)</t>
+  </si>
+  <si>
+    <t>S7</t>
+  </si>
+  <si>
+    <t>S8</t>
+  </si>
+  <si>
+    <t>0.2</t>
+  </si>
+  <si>
+    <t>Accessibilité RGAA + i18n + scalabilité (J4)</t>
+  </si>
+  <si>
+    <t>Préparation conformité et montée en charge</t>
+  </si>
+  <si>
+    <t>Amélioration performance et qualité</t>
+  </si>
+  <si>
+    <t>Évolution technique LLM (J2 - benchmark + ADR)</t>
+  </si>
+  <si>
+    <t>Intégration vue enseignant minimale (US-07)</t>
+  </si>
+  <si>
+    <t>Ajout besoins enseignant (J1 - Mme Lefèvre)</t>
+  </si>
+  <si>
+    <t>Stabilisation et corresction post-MVP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Livraison MVP étudiant </t>
+  </si>
+  <si>
+    <t>Départ/ initialisation backlog</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -225,44 +240,39 @@
       <sz val="16"/>
       <color rgb="FF1E1B4B"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="11"/>
       <color rgb="FF64748B"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
       <color rgb="FF4F46E5"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10.5"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="9"/>
       <color rgb="FF94A3B8"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF64748B"/>
-      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -270,6 +280,27 @@
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF64748B"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <strike/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -290,7 +321,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -313,11 +344,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD1D5DB"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD1D5DB"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -346,6 +388,8 @@
     <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -805,9 +849,9 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>'Burnup (projet)'!$A$5:$A$11</c:f>
+              <c:f>'Burnup (projet)'!$A$5:$A$13</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="9"/>
                 <c:pt idx="0">
                   <c:v>S0</c:v>
                 </c:pt>
@@ -828,6 +872,12 @@
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>S6</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>S7</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>S8</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -839,22 +889,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="7"/>
                 <c:pt idx="0">
+                  <c:v>41</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>41</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>60</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>80</c:v>
+                </c:pt>
+                <c:pt idx="4">
                   <c:v>100</c:v>
                 </c:pt>
-                <c:pt idx="1">
-                  <c:v>100</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>100</c:v>
-                </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="5">
                   <c:v>120</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>120</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>140</c:v>
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>140</c:v>
@@ -902,9 +952,9 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>'Burnup (projet)'!$A$5:$A$11</c:f>
+              <c:f>'Burnup (projet)'!$A$5:$A$13</c:f>
               <c:strCache>
-                <c:ptCount val="7"/>
+                <c:ptCount val="9"/>
                 <c:pt idx="0">
                   <c:v>S0</c:v>
                 </c:pt>
@@ -925,6 +975,12 @@
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>S6</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>S7</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>S8</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -939,22 +995,22 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>20</c:v>
+                  <c:v>41</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>42</c:v>
+                  <c:v>55</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>64</c:v>
+                  <c:v>75</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>86</c:v>
+                  <c:v>95</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>108</c:v>
+                  <c:v>115</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>128</c:v>
+                  <c:v>135</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1525,7 +1581,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -1574,7 +1630,7 @@
         <v>22</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
@@ -1673,7 +1729,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="8">
         <v>8</v>
       </c>
@@ -1685,7 +1741,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" s="8">
         <v>9</v>
       </c>
@@ -1697,7 +1753,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" s="8">
         <v>10</v>
       </c>
@@ -1709,12 +1765,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A21" s="3" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" s="11" t="s">
         <v>24</v>
       </c>
@@ -1723,7 +1779,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" s="11" t="s">
         <v>25</v>
       </c>
@@ -1732,7 +1788,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" s="11" t="s">
         <v>26</v>
       </c>
@@ -1741,7 +1797,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" s="11" t="s">
         <v>27</v>
       </c>
@@ -1749,6 +1805,9 @@
         <f>(B5-C19)/B5</f>
         <v>0.97499999999999998</v>
       </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F28" s="16"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1758,7 +1817,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
@@ -1798,161 +1857,186 @@
         <v>34</v>
       </c>
       <c r="B5" s="10">
-        <v>100</v>
+        <v>41</v>
       </c>
       <c r="C5" s="10">
         <v>0</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>35</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B6" s="10">
-        <v>100</v>
+        <v>41</v>
       </c>
       <c r="C6" s="10">
-        <v>20</v>
+        <v>41</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>50</v>
+        <v>60</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B7" s="10">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="C7" s="10">
-        <v>42</v>
+        <v>55</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B8" s="10">
-        <v>120</v>
+        <v>80</v>
       </c>
       <c r="C8" s="10">
-        <v>64</v>
+        <v>75</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B9" s="10">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="C9" s="10">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B10" s="10">
+        <v>120</v>
+      </c>
+      <c r="C10" s="10">
+        <v>115</v>
+      </c>
+      <c r="D10" s="14" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A11" s="17" t="s">
         <v>40</v>
-      </c>
-      <c r="B10" s="10">
-        <v>140</v>
-      </c>
-      <c r="C10" s="10">
-        <v>108</v>
-      </c>
-      <c r="D10" s="14" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A11" s="8" t="s">
-        <v>41</v>
       </c>
       <c r="B11" s="10">
         <v>140</v>
       </c>
       <c r="C11" s="10">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="D11" s="13" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A12" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="B12" s="10">
+        <v>155</v>
+      </c>
+      <c r="C12" s="10">
+        <v>150</v>
+      </c>
+      <c r="D12" s="13" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A13" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B13" s="10">
+        <v>194</v>
+      </c>
+      <c r="C13" s="10">
+        <v>189</v>
+      </c>
+      <c r="D13" s="13" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A13" s="3" t="s">
+    <row r="16" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A16" s="3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A17" s="11" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" s="11" t="s">
+      <c r="B17" s="8">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A18" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="B14" s="8">
-        <f>COUNTA(A5:A11)-1</f>
-        <v>6</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A15" s="11" t="s">
+      <c r="B18" s="8">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A19" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="B15" s="8">
-        <f>ROUND(C11/(COUNTA(A5:A11)-1),1)</f>
-        <v>21.3</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A16" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="B16" s="8">
+      <c r="B19" s="8">
         <f>B11</f>
         <v>140</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A17" s="11" t="s">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A20" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="B20" s="8">
+        <f>C11</f>
+        <v>135</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A21" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="B17" s="8">
-        <f>C11</f>
-        <v>128</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A18" s="11" t="s">
+      <c r="B21" s="8">
+        <f>B11-C11</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A22" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="B18" s="8">
-        <f>B11-C11</f>
-        <v>12</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A19" s="11" t="s">
+      <c r="B22" s="8" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A24" s="5" t="s">
         <v>48</v>
-      </c>
-      <c r="B19" s="8">
-        <f>ROUND((B11-C11)/(C11/(COUNTA(A5:A11)-1)),1)</f>
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A21" s="5" t="s">
-        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>